<commit_message>
Autónomos: panel «Antes de calcular» con avisos sobre las facturas importadas, cada uno con su acción para corregirlo
Módulo de dominio puro (importChecks) y testeado: facturas repetidas, fecha en un trimestre distinto del que dice la columna «Periodo/Trimestre», trimestres ya empezados sin ingresos o sin gastos, «Otros gastos» por encima del 30 %, modelo 130 importado que no cuadra con las facturas (ingresos y gastos deducibles acumulados, tolerancia 1 €), gastos al 0 % de IVA que no son cuota/sueldos/seguros/multas, rectificativas y facturas de otro año. Cada aviso abre la factura en la tabla de revisión (desplegándola y con el foco en su tipo de gasto) o lleva al trimestre.

El generador de ejemplos ponía «2T» a la factura de julio en la columna Periodo: corregido y regenerado el libro de ejemplo de emitidas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ejemplos-importacion/ejemplo-facturas-emitidas-2026.xlsx
+++ b/docs/ejemplos-importacion/ejemplo-facturas-emitidas-2026.xlsx
@@ -94,10 +94,10 @@
     <t xml:space="preserve">2026-006</t>
   </si>
   <si>
+    <t xml:space="preserve">3T</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3T</t>
   </si>
   <si>
     <t xml:space="preserve">2026-008</t>
@@ -437,7 +437,7 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
         <v>16</v>
@@ -446,7 +446,7 @@
         <v>46213</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
         <v>18</v>
@@ -475,7 +475,7 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
@@ -513,7 +513,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>

</xml_diff>